<commit_message>
Integrate Mocha 2 (Wande et al. 2026) into arid_humans
- add load_mocha() function to build_arid.py for reading and normalizing
  Mocha2_IsotopeData.xlsx
- mocha data: 8 individuals from Tarapaca Lowlands, Late Intermediate period
- δ13C range: -18.6 to -8‰ · δ15N range: 18.4 to 22.9‰
- integrate into humans table via --mocha flag; arid_humans grows from 2598 to
  2606 rows
- update arid_humans documentation: 2598 → 2606 rows
- rebuild all xlsx and reload package data

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/arid_sites.xlsx
+++ b/data-raw/arid_sites.xlsx
@@ -1477,7 +1477,7 @@
     <t>20 km south of Iquique</t>
   </si>
   <si>
-    <t>UpperTarapaca Valley</t>
+    <t>Mocha</t>
   </si>
   <si>
     <t>Middle Lluta Valley, Poconchile</t>
@@ -7241,13 +7241,13 @@
         <v>225</v>
       </c>
       <c r="B216">
-        <v>-19.832041</v>
+        <v>-19.81231</v>
       </c>
       <c r="C216">
-        <v>-69.296723</v>
+        <v>-69.28215</v>
       </c>
       <c r="D216">
-        <v>2274</v>
+        <v>1650</v>
       </c>
       <c r="E216" t="s">
         <v>487</v>
@@ -7256,7 +7256,7 @@
         <v>455</v>
       </c>
       <c r="G216" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="H216" t="s">
         <v>519</v>
@@ -7265,7 +7265,7 @@
         <v>519</v>
       </c>
       <c r="J216">
-        <v>1100</v>
+        <v>1250</v>
       </c>
       <c r="K216">
         <v>1450</v>

</xml_diff>

<commit_message>
Correct Mocha 2 altitude: 1650 → 2170 masl (Precordillera)
- update load_mocha() altitude from ~1,650 to 2,170 masl
- ecozone now correctly assigned as Precordillera (1700–3700 masl range)
- rebuild xlsx and reload package data

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/arid_sites.xlsx
+++ b/data-raw/arid_sites.xlsx
@@ -7247,7 +7247,7 @@
         <v>-69.28215</v>
       </c>
       <c r="D216">
-        <v>1650</v>
+        <v>2170</v>
       </c>
       <c r="E216" t="s">
         <v>487</v>
@@ -7256,7 +7256,7 @@
         <v>455</v>
       </c>
       <c r="G216" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="H216" t="s">
         <v>519</v>

</xml_diff>

<commit_message>
Fix Calate admin_region: Tarapaca → Antofagasta
- Add SITE_ADMIN_OVERRIDE dict for site-level corrections to admin_region
- Apply override in clean_table() and build_sites() to cover both sample
  tables and sites derived from the C14 database (Mendez-Quiros)
- All 13 Calate/* sites now correctly assigned to Antofagasta

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-raw/arid_sites.xlsx
+++ b/data-raw/arid_sites.xlsx
@@ -3369,7 +3369,7 @@
         <v>445</v>
       </c>
       <c r="F50" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G50" t="s">
         <v>511</v>
@@ -3398,7 +3398,7 @@
         <v>446</v>
       </c>
       <c r="F51" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G51" t="s">
         <v>511</v>
@@ -3415,7 +3415,7 @@
         <v>446</v>
       </c>
       <c r="F52" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G52" t="s">
         <v>511</v>
@@ -3432,7 +3432,7 @@
         <v>446</v>
       </c>
       <c r="F53" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G53" t="s">
         <v>511</v>
@@ -3449,7 +3449,7 @@
         <v>446</v>
       </c>
       <c r="F54" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G54" t="s">
         <v>511</v>
@@ -3466,7 +3466,7 @@
         <v>446</v>
       </c>
       <c r="F55" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G55" t="s">
         <v>511</v>
@@ -3483,7 +3483,7 @@
         <v>446</v>
       </c>
       <c r="F56" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G56" t="s">
         <v>511</v>
@@ -3500,7 +3500,7 @@
         <v>446</v>
       </c>
       <c r="F57" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G57" t="s">
         <v>511</v>
@@ -3517,7 +3517,7 @@
         <v>446</v>
       </c>
       <c r="F58" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G58" t="s">
         <v>511</v>
@@ -3534,7 +3534,7 @@
         <v>446</v>
       </c>
       <c r="F59" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G59" t="s">
         <v>511</v>
@@ -3551,7 +3551,7 @@
         <v>446</v>
       </c>
       <c r="F60" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G60" t="s">
         <v>511</v>
@@ -3568,7 +3568,7 @@
         <v>446</v>
       </c>
       <c r="F61" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G61" t="s">
         <v>511</v>
@@ -3585,7 +3585,7 @@
         <v>446</v>
       </c>
       <c r="F62" t="s">
-        <v>455</v>
+        <v>508</v>
       </c>
       <c r="G62" t="s">
         <v>511</v>

</xml_diff>